<commit_message>
feat(cronograma): integrar estrutura oficial da planilha F4A e suporte robusto a importacao Excel
</commit_message>
<xml_diff>
--- a/cronograma_oficial_4andar_2026.xlsx
+++ b/cronograma_oficial_4andar_2026.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Planejamento 2026" sheetId="1" r:id="rId1"/>
+    <sheet name="CRONOGRAMA e EQUIPE" sheetId="1" r:id="rId1"/>
+    <sheet name="2023 CRONOGRAMA" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,1399 +398,3067 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Data</v>
       </c>
       <c r="B1" t="str">
+        <v>B1 Manhã</v>
+      </c>
+      <c r="C1" t="str">
         <v>I2 Manhã</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
+        <v>B2 Manhã</v>
+      </c>
+      <c r="E1" t="str">
+        <v>I1 Manhã</v>
+      </c>
+      <c r="F1" t="str">
+        <v>B1 Tarde</v>
+      </c>
+      <c r="G1" t="str">
         <v>I1 Tarde</v>
       </c>
-      <c r="D1" t="str">
-        <v>B1 Manhã</v>
-      </c>
-      <c r="E1" t="str">
-        <v>B2 Manhã</v>
-      </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>B2 Tarde</v>
       </c>
-      <c r="G1" t="str">
-        <v>I1 Manhã</v>
-      </c>
-      <c r="H1" t="str">
-        <v>B1 Tarde</v>
+      <c r="I1" t="str">
+        <v>I2 Tarde</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sábado, 04/01</v>
+        <v>sábado, 03/01</v>
       </c>
       <c r="B2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="C2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="D2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="E2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="F2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="G2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="H2" t="str">
-        <v>Ano Novo - SEM AULA</v>
+        <v>SEM AULA - RECESSO</v>
+      </c>
+      <c r="I2" t="str">
+        <v>SEM AULA - RECESSO</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sábado, 11/01</v>
+        <v>sábado, 10/01</v>
       </c>
       <c r="B3" t="str">
-        <v>Esmeril Quebrado</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="C3" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="D3" t="str">
-        <v>Passo Básico</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="E3" t="str">
-        <v>Ritmo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="F3" t="str">
-        <v>Ritmo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="G3" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="H3" t="str">
-        <v>Passo Básico</v>
+        <v>SEM AULA - RECESSO</v>
+      </c>
+      <c r="I3" t="str">
+        <v>SEM AULA - RECESSO</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sábado, 18/01</v>
+        <v>sábado, 17/01</v>
       </c>
       <c r="B4" t="str">
-        <v>Esmeril Invertido</v>
+        <v>Passo Básico (Prof: BIA)</v>
       </c>
       <c r="C4" t="str">
-        <v>Banana c contra</v>
+        <v>Turma junta (Prof: DAVIDSON)</v>
       </c>
       <c r="D4" t="str">
-        <v>Xaxadinho</v>
+        <v>Início Módulo - Musicalidade (Prof: TONY)</v>
       </c>
       <c r="E4" t="str">
-        <v>Musicalidade</v>
+        <v>Sacada/Meia-lua (Prof: DAVIDSON)</v>
       </c>
       <c r="F4" t="str">
-        <v>Musicalidade</v>
+        <v>Passo Básico (Prof: MESSIAS)</v>
       </c>
       <c r="G4" t="str">
-        <v>Banana c contra</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H4" t="str">
-        <v>Xaxadinho</v>
+        <v>Passo de Cintura (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Trocadilho (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>sábado, 25/01</v>
+        <v>sábado, 24/01</v>
       </c>
       <c r="B5" t="str">
-        <v>Miudinho</v>
+        <v>Soltinho (Prof: BIA)</v>
       </c>
       <c r="C5" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
       <c r="D5" t="str">
-        <v>Deslocamento 1</v>
+        <v>Especial (Prof: TONY E JULY)</v>
       </c>
       <c r="E5" t="str">
-        <v>Breques</v>
+        <v>Sinistro (Prof: GÃO)</v>
       </c>
       <c r="F5" t="str">
-        <v>Breques</v>
+        <v>Meio Giro Trás/Frente (Aulão/Junto) (Prof: MESSIAS)</v>
       </c>
       <c r="G5" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H5" t="str">
-        <v>Deslocamento 1</v>
+        <v>Passo de Cintura (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Trocadilho inverso (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>sábado, 01/02</v>
+        <v>sábado, 31/01</v>
       </c>
       <c r="B6" t="str">
-        <v>Sacada com Pescada</v>
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: BIA)</v>
       </c>
       <c r="C6" t="str">
-        <v>Sinistro</v>
+        <v>Sequência de passo de perna + paulista (Prof: DAVIDSON)</v>
       </c>
       <c r="D6" t="str">
-        <v>Deslocamento 2</v>
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E6" t="str">
-        <v>Revisão Meio Giro</v>
+        <v>Sequência de caracol com avião (Prof: GÃO)</v>
       </c>
       <c r="F6" t="str">
-        <v>Revisão Meio Giro</v>
+        <v>Revisão passo simples, soltinho e meio giro (Prof: MESSIAS)</v>
       </c>
       <c r="G6" t="str">
-        <v>Sinistro</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H6" t="str">
-        <v>Deslocamento 2</v>
+        <v>Revisão passo cintura e início esmeril (Prof: TAZ)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sábado, 08/02</v>
+        <v>sábado, 07/02</v>
       </c>
       <c r="B7" t="str">
-        <v>Sacada com arrasto</v>
+        <v>Abertura soltinho e giro simples (Prof: BIA)</v>
       </c>
       <c r="C7" t="str">
-        <v>Avião c contra</v>
+        <v>Avião invertido + contratempo (Prof: DAVIDSON)</v>
       </c>
       <c r="D7" t="str">
-        <v>Ritmos</v>
+        <v>Giro-giro (Prof: GÃO)</v>
       </c>
       <c r="E7" t="str">
-        <v>Pega-Pega</v>
+        <v>Avião com contratempos (Prof: GÃO)</v>
       </c>
       <c r="F7" t="str">
-        <v>Pega-Pega</v>
+        <v>Meio giro (Prof: MESSIAS)</v>
       </c>
       <c r="G7" t="str">
-        <v>Avião c contra</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H7" t="str">
-        <v>Ritmos</v>
+        <v>Esmeril junto (Prof: TAZ)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Condução do Paulista (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>sábado, 15/02</v>
+        <v>sábado, 14/02</v>
       </c>
       <c r="B8" t="str">
-        <v>Leque</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="C8" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="D8" t="str">
-        <v>Giro Completo</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="E8" t="str">
-        <v>Giro Giro</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="F8" t="str">
-        <v>Giro Giro</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="G8" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>SEM AULA - CARNAVAL</v>
       </c>
       <c r="H8" t="str">
-        <v>Giro Completo</v>
+        <v>SEM AULA - CARNAVAL</v>
+      </c>
+      <c r="I8" t="str">
+        <v>SEM AULA - CARNAVAL</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sábado, 22/02</v>
+        <v>sábado, 21/02</v>
       </c>
       <c r="B9" t="str">
-        <v>Push and Pull</v>
+        <v>Troca de peso e passo básico (Prof: BIA)</v>
       </c>
       <c r="C9" t="str">
-        <v>Basquete com Contra</v>
+        <v>Sequência das últimas aulas (Prof: DAVIDSON)</v>
       </c>
       <c r="D9" t="str">
-        <v>Giro Simples</v>
+        <v>Banana banana (Prof: TONY)</v>
       </c>
       <c r="E9" t="str">
-        <v>Caracol</v>
+        <v>Avião + contratempo (Prof: TAZ E BIA)</v>
       </c>
       <c r="F9" t="str">
-        <v>Caracol</v>
+        <v>Passo básico e meio-giros (Prof: BIA)</v>
       </c>
       <c r="G9" t="str">
-        <v>Basquete com Contra</v>
+        <v>Giro-giro com contratempo (Prof: TAZ E BIA)</v>
       </c>
       <c r="H9" t="str">
-        <v>Giro Simples</v>
+        <v>Esmeril junto (Prof: TAZ E JULY)</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Movimentações do paulista (saída do pião/meio giro trás e do meio invertido trás) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>sábado, 01/03</v>
+        <v>sábado, 28/02</v>
       </c>
       <c r="B10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Postura e Ritmo (Prof: BIA)</v>
       </c>
       <c r="C10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
       <c r="D10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Giro completo trás/frente (junto) (Prof: GÃO)</v>
       </c>
       <c r="F10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Postura e Ritmo (Prof: MESSIAS)</v>
       </c>
       <c r="G10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Giro completo trás/frente (junto) (Prof: GÃO)</v>
       </c>
       <c r="H10" t="str">
-        <v>Carnaval - SEM AULA</v>
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sábado, 08/03</v>
+        <v>sábado, 07/03</v>
       </c>
       <c r="B11" t="str">
-        <v>Paulista Titanic</v>
+        <v>Giro da dama e giro cavalheiro (Prof: JULY)</v>
       </c>
       <c r="C11" t="str">
-        <v>Esmeril aberto</v>
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
       <c r="D11" t="str">
-        <v>Giro do Condutor</v>
+        <v>banana-banana (Prof: DAVIDSON)</v>
       </c>
       <c r="E11" t="str">
-        <v>Avião</v>
+        <v>turma junta (Prof: DAVIDSON)</v>
       </c>
       <c r="F11" t="str">
-        <v>Avião</v>
+        <v>básico e meio-giro (Prof: JULY)</v>
       </c>
       <c r="G11" t="str">
-        <v>Esmeril aberto</v>
+        <v>chuveirinho com contratempo + banana com contratempo (Prof: TAZ)</v>
       </c>
       <c r="H11" t="str">
-        <v>Giro do Condutor</v>
+        <v>Início contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sábado, 15/03</v>
+        <v>sábado, 14/03</v>
       </c>
       <c r="B12" t="str">
-        <v>Contra 9 tempos</v>
+        <v>GIRO SIMPLES (Prof: BIA)</v>
       </c>
       <c r="C12" t="str">
-        <v>Esmeril unilateral</v>
+        <v>Sequencia com contratempo de 7 (Prof: DAVIDSON)</v>
       </c>
       <c r="D12" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>Avião (Prof: TONY)</v>
       </c>
       <c r="E12" t="str">
-        <v>Assalto</v>
+        <v>giro-giro com contratempo (Prof: GÃO)</v>
       </c>
       <c r="F12" t="str">
-        <v>Assalto</v>
+        <v>Postura + passos iniciais (Prof: MESSIAS)</v>
       </c>
       <c r="G12" t="str">
-        <v>Esmeril unilateral</v>
+        <v>contratempo de 5 tempos + 7 tempos (Prof: GÃO)</v>
       </c>
       <c r="H12" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>CONTRATEMPO condução (Prof: TAZ E JULY)</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Variação de Avião (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sábado, 22/03</v>
+        <v>sábado, 21/03</v>
       </c>
       <c r="B13" t="str">
-        <v>Banana 9 tempos</v>
+        <v>xaxadinho; chuveirinho (Prof: GÃO)</v>
       </c>
       <c r="C13" t="str">
-        <v>Firula</v>
+        <v>Introdução cretinagem (Prof: DAVIDSON)</v>
       </c>
       <c r="D13" t="str">
-        <v>Chuveirinho</v>
+        <v>Revisão (Prof: TONY)</v>
       </c>
       <c r="E13" t="str">
-        <v>Banana Banana</v>
+        <v>Passo de Cintura (+Variações com contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F13" t="str">
-        <v>Banana Banana</v>
+        <v>Giro simples (Prof: JULY)</v>
       </c>
       <c r="G13" t="str">
-        <v>Firula</v>
+        <v>sinistro com contratempo + banana invertida (Prof: GÃO)</v>
       </c>
       <c r="H13" t="str">
-        <v>Chuveirinho</v>
+        <v>contratempo (Prof: TONY)</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Contratempos duplos (sinistro e 1ª evolução do sinistro) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sábado, 29/03</v>
+        <v>sábado, 28/03</v>
       </c>
       <c r="B14" t="str">
-        <v>Chuveirinho 9 tempos</v>
+        <v>Meios giros/Nivelamento (Prof: GÃO E BIA)</v>
       </c>
       <c r="C14" t="str">
-        <v>Musicalidade</v>
+        <v>Giro completo invertido + pião invertido (Prof: DAVIDSON)</v>
       </c>
       <c r="D14" t="str">
-        <v>Manivela</v>
+        <v>Início de cintura (Prof: TONY)</v>
       </c>
       <c r="E14" t="str">
-        <v>Combinações de Passos</v>
+        <v>Sacada/Meia-lua (Prof: GÃO E BIA)</v>
       </c>
       <c r="F14" t="str">
-        <v>Combinações de Passos</v>
+        <v>GIro simples (Prof: MESSIAS)</v>
       </c>
       <c r="G14" t="str">
-        <v>Musicalidade</v>
+        <v>Sacada/Meia-lua (Prof: GÃO)</v>
       </c>
       <c r="H14" t="str">
-        <v>Manivela</v>
+        <v>Caracol com contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Variação de Banana (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sábado, 05/04</v>
+        <v>sábado, 04/04</v>
       </c>
       <c r="B15" t="str">
-        <v>Sinistro 9 e 11</v>
+        <v>Início Módulo (Prof: BIA)</v>
       </c>
       <c r="C15" t="str">
-        <v>Sacada e Pendulo</v>
+        <v>Sacada com a perna esquerda (Prof: DAVIDSON)</v>
       </c>
       <c r="D15" t="str">
-        <v>Caracol</v>
+        <v>passo de cintura (Prof: TONY)</v>
       </c>
       <c r="E15" t="str">
-        <v>Cintura</v>
+        <v>Pêndulo/Ciscada (Prof: GÃO)</v>
       </c>
       <c r="F15" t="str">
-        <v>Cintura</v>
+        <v>Giro simples (Prof: JULY)</v>
       </c>
       <c r="G15" t="str">
-        <v>Sacada e Pendulo</v>
+        <v>Introdução Paulista (Prof: GÃO)</v>
       </c>
       <c r="H15" t="str">
-        <v>Caracol</v>
+        <v>REVISÃO (Prof: TAZ)</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Variação de Passos de Cintura (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>sábado, 12/04</v>
+        <v>sábado, 11/04</v>
       </c>
       <c r="B16" t="str">
-        <v>Avião Invertido</v>
+        <v>Início Módulo - Peso e contrapeso (Prof: GÃO E BIA)</v>
       </c>
       <c r="C16" t="str">
-        <v>Sacada Meia Lua</v>
+        <v>Sacada de letra (Prof: DAVIDSON)</v>
       </c>
       <c r="D16" t="str">
-        <v>Revisão</v>
+        <v>passo de cintura (Prof: TONY)</v>
       </c>
       <c r="E16" t="str">
-        <v>Volta ao Mundo</v>
+        <v>Introdução ao Paulista (Prof: GÃO)</v>
       </c>
       <c r="F16" t="str">
-        <v>Volta ao Mundo</v>
+        <v>Passo Básico (Prof: MESSIAS)</v>
       </c>
       <c r="G16" t="str">
-        <v>Sacada Meia Lua</v>
+        <v>Paulista com invertido atrás (Prof: GÃO)</v>
       </c>
       <c r="H16" t="str">
-        <v>Revisão</v>
+        <v>Revisão Nivelamento (Prof: TAZ)</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Combinação de Cintura com Peões (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>sábado, 19/04</v>
+        <v>sábado, 18/04</v>
       </c>
       <c r="B17" t="str">
-        <v>Beyblade 9</v>
+        <v>Meio-giro dançando junto (Prof: GÃO E BIA)</v>
       </c>
       <c r="C17" t="str">
-        <v>Caminhada e travada</v>
+        <v>Sequencia de sacada de esquerda (Prof: DAVIDSON)</v>
       </c>
       <c r="D17" t="str">
-        <v>Nivelamento</v>
+        <v>Passo de cintura saindo no invertido (Prof: TONY E JULY)</v>
       </c>
       <c r="E17" t="str">
-        <v>Combinação de Cintura</v>
+        <v>Paulista (Prof: GÃO E BIA)</v>
       </c>
       <c r="F17" t="str">
-        <v>Combinação de Cintura</v>
+        <v>Giro do cavalheiro (Prof: MESSIAS)</v>
       </c>
       <c r="G17" t="str">
-        <v>Caminhada e travada</v>
+        <v>Paulista (Prof: GÃO)</v>
       </c>
       <c r="H17" t="str">
-        <v>Nivelamento</v>
+        <v>Revisão e Nivelamento (Prof: TAZ)</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Giros invertidos completos (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>sábado, 26/04</v>
+        <v>sábado, 25/04</v>
       </c>
       <c r="B18" t="str">
-        <v>Giro Simples 9 e 11</v>
+        <v>Troca de peso (Prof: BIA)</v>
       </c>
       <c r="C18" t="str">
-        <v>Paulista</v>
+        <v>Aula livre (Prof: DAVIDSON)</v>
       </c>
       <c r="D18" t="str">
-        <v>Passo Básico</v>
+        <v>Ritmo (Prof: TONY)</v>
       </c>
       <c r="E18" t="str">
-        <v>Esmeril Fechado</v>
+        <v>Nivelamento + Paulista (Prof: GÃO)</v>
       </c>
       <c r="F18" t="str">
-        <v>Esmeril Fechado</v>
+        <v>Troca de peso (Prof: MESSIAS)</v>
       </c>
       <c r="G18" t="str">
-        <v>Paulista</v>
+        <v>Banana finalizando com paulista (Prof: GÃO)</v>
       </c>
       <c r="H18" t="str">
-        <v>Passo Básico</v>
+        <v>Aula junto com o Básico 1 (Prof: TAZ)</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Esmeril unilateral (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>sábado, 03/05</v>
+        <v>sábado, 02/05</v>
       </c>
       <c r="B19" t="str">
-        <v>Basquete 11</v>
+        <v>Revisão (Prof: BIA)</v>
       </c>
       <c r="C19" t="str">
-        <v>Combinação de Paulista</v>
+        <v>bêbado (Prof: DAVIDSON)</v>
       </c>
       <c r="D19" t="str">
-        <v>Xaxadinho</v>
+        <v>ESMERIL JUNTO (Prof: TONY E JULY)</v>
       </c>
       <c r="E19" t="str">
-        <v>Práticas dançantes</v>
+        <v>PAULISTA COM INVERTIDO TRÁS (Prof: GÃO E BIA)</v>
       </c>
       <c r="F19" t="str">
-        <v>Práticas dançantes</v>
+        <v>Variação do giro simples (Prof: JULY)</v>
       </c>
       <c r="G19" t="str">
-        <v>Combinação de Paulista</v>
+        <v>introdução ao esmeril (Prof: GÃO E JULY)</v>
       </c>
       <c r="H19" t="str">
-        <v>Xaxadinho</v>
+        <v>Revisão (Prof: TAZ)</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Especial (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>sábado, 10/05</v>
+        <v>sábado, 09/05</v>
       </c>
       <c r="B20" t="str">
-        <v>Esmeril Quebrado</v>
+        <v>variações de giro simples (Prof: BIA)</v>
       </c>
       <c r="C20" t="str">
-        <v>Pião</v>
+        <v>paulista (Prof: DAVIDSON)</v>
       </c>
       <c r="D20" t="str">
-        <v>Deslocamento 1</v>
+        <v>esmeril junto (Prof: TONY)</v>
       </c>
       <c r="E20" t="str">
-        <v>Introdução Contratempo</v>
+        <v>Início Módulo - Paulista com invertido (Prof: GÃO E BIA)</v>
       </c>
       <c r="F20" t="str">
-        <v>Introdução Contratempo</v>
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G20" t="str">
-        <v>Pião</v>
+        <v>esmeril (variações) (Prof: GÃO)</v>
       </c>
       <c r="H20" t="str">
-        <v>Deslocamento 1</v>
+        <v>Musicalidade (Prof: TAZ)</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Turma junta (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>sábado, 17/05</v>
+        <v>sábado, 16/05</v>
       </c>
       <c r="B21" t="str">
-        <v>Esmeril Invertido</v>
+        <v>Postura e Ritmo (Prof: BIA)</v>
       </c>
       <c r="C21" t="str">
-        <v>Revisão</v>
+        <v>Trocadilho (Prof: DAVIDSON)</v>
       </c>
       <c r="D21" t="str">
-        <v>Deslocamento 2</v>
+        <v>esmeril (Prof: DAVIDSON)</v>
       </c>
       <c r="E21" t="str">
-        <v>Caracol c Contra</v>
+        <v>Introdução esmeril aberto (Prof: GÃO E BIA)</v>
       </c>
       <c r="F21" t="str">
-        <v>Caracol c Contra</v>
+        <v>Postura e Ritmo (Prof: MESSIAS)</v>
       </c>
       <c r="G21" t="str">
-        <v>Revisão</v>
+        <v>esmeril; introdução pião (Prof: GÃO)</v>
       </c>
       <c r="H21" t="str">
-        <v>Deslocamento 2</v>
+        <v>NIVELAMENTO (Prof: TAZ)</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Trocadilho (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>sábado, 24/05</v>
+        <v>sábado, 23/05</v>
       </c>
       <c r="B22" t="str">
-        <v>Miudinho</v>
+        <v>REVISÃO (Prof: BIA)</v>
       </c>
       <c r="C22" t="str">
-        <v>Nivelamento</v>
+        <v>Trocadilho inverso (Prof: DAVIDSON)</v>
       </c>
       <c r="D22" t="str">
-        <v>Ritmos</v>
+        <v>cobrinha (Prof: TONY E JULY)</v>
       </c>
       <c r="E22" t="str">
-        <v>Conduções de Contra</v>
+        <v>esmeril abberto (Prof: GÃO)</v>
       </c>
       <c r="F22" t="str">
-        <v>Conduções de Contra</v>
+        <v>manivela (Prof: MESSIAS)</v>
       </c>
       <c r="G22" t="str">
-        <v>Nivelamento</v>
+        <v>pião (Prof: GÃO)</v>
       </c>
       <c r="H22" t="str">
-        <v>Ritmos</v>
+        <v>invertido (Prof: TAZ)</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Trocadilho inverso (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>sábado, 31/05</v>
+        <v>sábado, 30/05</v>
       </c>
       <c r="B23" t="str">
-        <v>Sacada com Pescada</v>
+        <v>Nivelamento (Prof: BIA)</v>
       </c>
       <c r="C23" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
       <c r="D23" t="str">
-        <v>Giro Completo</v>
+        <v>Contratempo introdução (Prof: TONY E JULY)</v>
       </c>
       <c r="E23" t="str">
-        <v>Contra do Passo Básico</v>
+        <v>esmeril variações (Prof: GÃO)</v>
       </c>
       <c r="F23" t="str">
-        <v>Contra do Passo Básico</v>
+        <v>nivelamento (Prof: MESSIAS)</v>
       </c>
       <c r="G23" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>pião (Prof: GÃO)</v>
       </c>
       <c r="H23" t="str">
-        <v>Giro Completo</v>
+        <v>revisão (Prof: TAZ)</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>sábado, 07/06</v>
+        <v>sábado, 06/06</v>
       </c>
       <c r="B24" t="str">
-        <v>Sacada com arrasto</v>
+        <v>Chameguinho (Aulão) (Prof: BIA)</v>
       </c>
       <c r="C24" t="str">
-        <v>Banana c contra</v>
+        <v>Condução do Paulista (Prof: DAVIDSON)</v>
       </c>
       <c r="D24" t="str">
-        <v>Giro Simples</v>
+        <v>contratempo (Prof: TONY)</v>
       </c>
       <c r="E24" t="str">
-        <v>Combinações de Contra</v>
+        <v>técnicas de esmeril (Prof: BIA)</v>
       </c>
       <c r="F24" t="str">
-        <v>Combinações de Contra</v>
+        <v>Chameguinho (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G24" t="str">
-        <v>Banana c contra</v>
+        <v>técnicas de esmeril (Prof: BIA)</v>
       </c>
       <c r="H24" t="str">
-        <v>Giro Simples</v>
+        <v>Caminhada Esquerda/Direita (Prof: TAZ)</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Condução do Paulista (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>sábado, 14/06</v>
+        <v>sábado, 13/06</v>
       </c>
       <c r="B25" t="str">
-        <v>Leque</v>
+        <v>Especial (Prof: BIA)</v>
       </c>
       <c r="C25" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>Movimentações do paulista (saída do pião/meio giro trás e do meio invertido trás) (Prof: DAVIDSON)</v>
       </c>
       <c r="D25" t="str">
-        <v>Giro do Condutor</v>
+        <v>contratempo (Prof: TONY)</v>
       </c>
       <c r="E25" t="str">
-        <v>Revisão</v>
+        <v>I1 e I2 Pião (Prof: GÃO E BIA)</v>
       </c>
       <c r="F25" t="str">
-        <v>Revisão</v>
+        <v>manivela, giro dama e cavalheiro, variações (Prof: MESSIAS)</v>
       </c>
       <c r="G25" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>pião invertido (Prof: GÃO)</v>
       </c>
       <c r="H25" t="str">
-        <v>Giro do Condutor</v>
+        <v>combo de giro (Prof: TAZ)</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Movimentações do paulista (saída do pião/meio giro trás e do meio invertido trás) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>sábado, 21/06</v>
+        <v>sábado, 20/06</v>
       </c>
       <c r="B26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="C26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="D26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="E26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="F26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="G26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
       <c r="H26" t="str">
-        <v>São João - SEM AULA</v>
+        <v>SEM AULA - SÃO JOÃO</v>
+      </c>
+      <c r="I26" t="str">
+        <v>SEM AULA - SÃO JOÃO</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>sábado, 28/06</v>
+        <v>sábado, 27/06</v>
       </c>
       <c r="B27" t="str">
-        <v>Push and Pull</v>
+        <v>Turma Junta (Prof: BIA)</v>
       </c>
       <c r="C27" t="str">
-        <v>Sinistro</v>
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
       <c r="D27" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>contratempo (Prof: TONY E JULY)</v>
       </c>
       <c r="E27" t="str">
-        <v>Nivelamento</v>
+        <v>pião (Prof: GÃO)</v>
       </c>
       <c r="F27" t="str">
-        <v>Nivelamento</v>
+        <v>giro do cavalheiro (Prof: MESSIAS)</v>
       </c>
       <c r="G27" t="str">
-        <v>Sinistro</v>
+        <v>pião + contratempo (Prof: GÃO)</v>
       </c>
       <c r="H27" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>banana-banana (Prof: TAZ)</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>sábado, 05/07</v>
+        <v>sábado, 04/07</v>
       </c>
       <c r="B28" t="str">
-        <v>Paulista Titanic</v>
+        <v>Passo Básico (Prof: BIA)</v>
       </c>
       <c r="C28" t="str">
-        <v>Avião c contra</v>
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
       <c r="D28" t="str">
-        <v>Chuveirinho</v>
+        <v>contratempo (Prof: TONY E JULY)</v>
       </c>
       <c r="E28" t="str">
-        <v>Ritmo</v>
+        <v>pião (Prof: GÃO)</v>
       </c>
       <c r="F28" t="str">
-        <v>Ritmo</v>
+        <v>Passo Básico (Prof: MESSIAS)</v>
       </c>
       <c r="G28" t="str">
-        <v>Avião c contra</v>
+        <v>pião com travada (Prof: GÃO)</v>
       </c>
       <c r="H28" t="str">
-        <v>Chuveirinho</v>
+        <v>avião (Prof: TAZ)</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>sábado, 12/07</v>
+        <v>sábado, 11/07</v>
       </c>
       <c r="B29" t="str">
-        <v>Contra 9 tempos</v>
+        <v>Início Módulo - Soltinho (Prof: BIA)</v>
       </c>
       <c r="C29" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>Variação de Avião (Prof: DAVIDSON)</v>
       </c>
       <c r="D29" t="str">
-        <v>Manivela</v>
+        <v>Esmeril junto (Prof: TONY E JULY)</v>
       </c>
       <c r="E29" t="str">
-        <v>Musicalidade</v>
+        <v>Pêndulo/Ciscada (Prof: GÃO)</v>
       </c>
       <c r="F29" t="str">
-        <v>Musicalidade</v>
+        <v>Soltinho (Prof: MESSIAS)</v>
       </c>
       <c r="G29" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>Pêndulo/Ciscada (Prof: GÃO)</v>
       </c>
       <c r="H29" t="str">
-        <v>Manivela</v>
+        <v>Esmeril junto (Prof: TAZ)</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Variação de Avião (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>sábado, 19/07</v>
+        <v>sábado, 18/07</v>
       </c>
       <c r="B30" t="str">
-        <v>Banana 9 tempos</v>
+        <v>Troca de peso (Prof: BIA)</v>
       </c>
       <c r="C30" t="str">
-        <v>Basquete com Contra</v>
+        <v>Contratempos duplos (sinistro e 1ª evolução do sinistro) (Prof: DAVIDSON)</v>
       </c>
       <c r="D30" t="str">
-        <v>Caracol</v>
+        <v>Especial (Prof: TONY E JULY)</v>
       </c>
       <c r="E30" t="str">
-        <v>Breques</v>
+        <v>pião (Prof: GÃO)</v>
       </c>
       <c r="F30" t="str">
-        <v>Breques</v>
+        <v>Início Módulo - Troca de peso (Prof: MESSIAS)</v>
       </c>
       <c r="G30" t="str">
-        <v>Basquete com Contra</v>
+        <v>sacada de perna (Prof: GÃO)</v>
       </c>
       <c r="H30" t="str">
-        <v>Caracol</v>
+        <v>Início Módulo - Especial (Prof: TAZ)</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Contratempos duplos (sinistro e 1ª evolução do sinistro) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>sábado, 26/07</v>
+        <v>sábado, 25/07</v>
       </c>
       <c r="B31" t="str">
-        <v>Chuveirinho 9 tempos</v>
+        <v>peso e contrapeso (Prof: BIA)</v>
       </c>
       <c r="C31" t="str">
-        <v>Esmeril aberto</v>
+        <v>Variação de Banana (Prof: DAVIDSON)</v>
       </c>
       <c r="D31" t="str">
-        <v>Revisão</v>
+        <v>contratempo (Prof: TONY)</v>
       </c>
       <c r="E31" t="str">
-        <v>Revisão Meio Giro</v>
+        <v>Turma Junta (Prof: GÃO)</v>
       </c>
       <c r="F31" t="str">
-        <v>Revisão Meio Giro</v>
+        <v>Meio Giro Trás/Frente (Aulão/Junto) (Prof: MESSIAS)</v>
       </c>
       <c r="G31" t="str">
-        <v>Esmeril aberto</v>
+        <v>Turma Junta (Prof: GÃO)</v>
       </c>
       <c r="H31" t="str">
-        <v>Revisão</v>
+        <v>Turma Junta (Prof: TAZ)</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Variação de Banana (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>sábado, 02/08</v>
+        <v>sábado, 01/08</v>
       </c>
       <c r="B32" t="str">
-        <v>Sinistro 9 e 11</v>
+        <v>musicalidade (Prof: BIA)</v>
       </c>
       <c r="C32" t="str">
-        <v>Esmeril unilateral</v>
+        <v>- (Prof: DAVIDSON)</v>
       </c>
       <c r="D32" t="str">
-        <v>Nivelamento</v>
+        <v>contratempo (Prof: TONY E JULY)</v>
       </c>
       <c r="E32" t="str">
-        <v>Pega-Pega</v>
+        <v>pião com travada (Prof: GÃO)</v>
       </c>
       <c r="F32" t="str">
-        <v>Pega-Pega</v>
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G32" t="str">
-        <v>Esmeril unilateral</v>
+        <v>caminhada e travada (Prof: GÃO)</v>
       </c>
       <c r="H32" t="str">
-        <v>Nivelamento</v>
+        <v>Meio Giro Invertido Trás/Frente (Aulão/Junto) (Prof: TAZ)</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Variação de Passos de Cintura (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>sábado, 09/08</v>
+        <v>sábado, 08/08</v>
       </c>
       <c r="B33" t="str">
-        <v>Avião Invertido</v>
+        <v>Postura e Ritmo (Prof: BIA)</v>
       </c>
       <c r="C33" t="str">
-        <v>Firula</v>
+        <v>Combinação de Cintura com Peões (Prof: DAVIDSON)</v>
       </c>
       <c r="D33" t="str">
-        <v>Passo Básico</v>
+        <v>Avião (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E33" t="str">
-        <v>Giro Giro</v>
+        <v>Sinistro (Prof: GÃO)</v>
       </c>
       <c r="F33" t="str">
-        <v>Giro Giro</v>
+        <v>Postura e Ritmo (Prof: MESSIAS)</v>
       </c>
       <c r="G33" t="str">
-        <v>Firula</v>
+        <v>Sinistro (Prof: GÃO)</v>
       </c>
       <c r="H33" t="str">
-        <v>Passo Básico</v>
+        <v>Avião (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Combinação de Cintura com Peões (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>sábado, 16/08</v>
+        <v>sábado, 15/08</v>
       </c>
       <c r="B34" t="str">
-        <v>Beyblade 9</v>
+        <v>Giro Simples Cavalheiro/Dama (Prof: BIA)</v>
       </c>
       <c r="C34" t="str">
-        <v>Musicalidade</v>
+        <v>Giros invertidos completos (Prof: DAVIDSON)</v>
       </c>
       <c r="D34" t="str">
-        <v>Xaxadinho</v>
+        <v>Musicalidade (Prof: TONY E JULY)</v>
       </c>
       <c r="E34" t="str">
-        <v>Caracol</v>
+        <v>Contratempo (Prof: GÃO)</v>
       </c>
       <c r="F34" t="str">
-        <v>Caracol</v>
+        <v>Giro Simples Cavalheiro/Dama (Prof: MESSIAS)</v>
       </c>
       <c r="G34" t="str">
-        <v>Musicalidade</v>
+        <v>Contratempo (Prof: GÃO)</v>
       </c>
       <c r="H34" t="str">
-        <v>Xaxadinho</v>
+        <v>Musicalidade (Prof: TAZ)</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Giros invertidos completos (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>sábado, 23/08</v>
+        <v>sábado, 22/08</v>
       </c>
       <c r="B35" t="str">
-        <v>Giro Simples 9 e 11</v>
+        <v>Peso e Contrapeso (Prof: BIA)</v>
       </c>
       <c r="C35" t="str">
-        <v>Sacada e Pendulo</v>
+        <v>Esmeril unilateral (Prof: DAVIDSON)</v>
       </c>
       <c r="D35" t="str">
-        <v>Deslocamento 1</v>
+        <v>invertido (Prof: TONY)</v>
       </c>
       <c r="E35" t="str">
-        <v>Avião</v>
+        <v>caminhada + variações (Prof: GÃO E BIA)</v>
       </c>
       <c r="F35" t="str">
-        <v>Avião</v>
+        <v>- (Prof: MESSIAS)</v>
       </c>
       <c r="G35" t="str">
-        <v>Sacada e Pendulo</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H35" t="str">
-        <v>Deslocamento 1</v>
+        <v>Banana (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Esmeril unilateral (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>sábado, 30/08</v>
+        <v>sábado, 29/08</v>
       </c>
       <c r="B36" t="str">
-        <v>Basquete 11</v>
+        <v>Chameguinho (Aulão) (Prof: BIA)</v>
       </c>
       <c r="C36" t="str">
-        <v>Sacada Meia Lua</v>
+        <v>Especial (Prof: DAVIDSON)</v>
       </c>
       <c r="D36" t="str">
-        <v>Deslocamento 2</v>
+        <v>Chuveirinho (+Variações sem Contratempo (Prof: TONY E JULY)</v>
       </c>
       <c r="E36" t="str">
-        <v>Assalto</v>
+        <v>Banana (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F36" t="str">
-        <v>Assalto</v>
+        <v>Chameguinho (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G36" t="str">
-        <v>Sacada Meia Lua</v>
+        <v>Banana (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H36" t="str">
-        <v>Deslocamento 2</v>
+        <v>início de contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Especial (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>sábado, 06/09</v>
+        <v>sábado, 05/09</v>
       </c>
       <c r="B37" t="str">
-        <v>Esmeril Quebrado</v>
+        <v>Especial (Prof: BIA)</v>
       </c>
       <c r="C37" t="str">
-        <v>Caminhada e travada</v>
+        <v>Turma junta (Prof: DAVIDSON)</v>
       </c>
       <c r="D37" t="str">
-        <v>Ritmos</v>
+        <v>invertido (Prof: TONY E JULY)</v>
       </c>
       <c r="E37" t="str">
-        <v>Banana Banana</v>
+        <v>breck (Prof: GÃO)</v>
       </c>
       <c r="F37" t="str">
-        <v>Banana Banana</v>
+        <v>Especial (Prof: MESSIAS)</v>
       </c>
       <c r="G37" t="str">
-        <v>Caminhada e travada</v>
+        <v>Giro completo trás/frente (junto) (Prof: GÃO)</v>
       </c>
       <c r="H37" t="str">
-        <v>Ritmos</v>
+        <v>contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Turma junta (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>sábado, 13/09</v>
+        <v>sábado, 12/09</v>
       </c>
       <c r="B38" t="str">
-        <v>Esmeril Invertido</v>
+        <v>Turma Junta (Prof: BIA)</v>
       </c>
       <c r="C38" t="str">
-        <v>Paulista</v>
+        <v>Trocadilho (Prof: DAVIDSON)</v>
       </c>
       <c r="D38" t="str">
-        <v>Giro Completo</v>
+        <v>Caminhada Esquerda/Direita (Prof: TONY E JULY)</v>
       </c>
       <c r="E38" t="str">
-        <v>Combinações de Passos</v>
+        <v>Chuveirinho (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F38" t="str">
-        <v>Combinações de Passos</v>
+        <v>Turma Junta (Prof: MESSIAS)</v>
       </c>
       <c r="G38" t="str">
-        <v>Paulista</v>
+        <v>Chuveirinho (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H38" t="str">
-        <v>Giro Completo</v>
+        <v>Caminhada Esquerda/Direita (Prof: TAZ)</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Trocadilho (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>sábado, 20/09</v>
+        <v>sábado, 19/09</v>
       </c>
       <c r="B39" t="str">
-        <v>Miudinho</v>
+        <v>Passo Básico (Prof: BIA)</v>
       </c>
       <c r="C39" t="str">
-        <v>Combinação de Paulista</v>
+        <v>Trocadilho inverso (Prof: DAVIDSON)</v>
       </c>
       <c r="D39" t="str">
-        <v>Giro Simples</v>
+        <v>Xaxadinho (Aulão) (Prof: TONY E JULY)</v>
       </c>
       <c r="E39" t="str">
-        <v>Cintura</v>
+        <v>Giro Giro – Giro Gira (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F39" t="str">
-        <v>Cintura</v>
+        <v>Passo Básico (Prof: MESSIAS)</v>
       </c>
       <c r="G39" t="str">
-        <v>Combinação de Paulista</v>
+        <v>Giro Giro – Giro Gira (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H39" t="str">
-        <v>Giro Simples</v>
+        <v>Xaxadinho (Aulão) (Prof: TAZ)</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Trocadilho inverso (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>sábado, 27/09</v>
+        <v>sábado, 26/09</v>
       </c>
       <c r="B40" t="str">
-        <v>Sacada com Pescada</v>
+        <v>Soltinho (Prof: BIA)</v>
       </c>
       <c r="C40" t="str">
-        <v>Pião</v>
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
       <c r="D40" t="str">
-        <v>Giro do Condutor</v>
+        <v>Xaxadinho (junto) (Prof: TONY E JULY)</v>
       </c>
       <c r="E40" t="str">
-        <v>Volta ao Mundo</v>
+        <v>Passo de Cintura (+Variações com contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F40" t="str">
-        <v>Volta ao Mundo</v>
+        <v>Soltinho (Prof: MESSIAS)</v>
       </c>
       <c r="G40" t="str">
-        <v>Pião</v>
+        <v>Passo de Cintura (+Variações com contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H40" t="str">
-        <v>Giro do Condutor</v>
+        <v>Xaxadinho (junto) (Prof: TAZ)</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Passo de perna (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>sábado, 04/10</v>
+        <v>sábado, 03/10</v>
       </c>
       <c r="B41" t="str">
-        <v>Sacada com arrasto</v>
+        <v>Início Módulo - Troca de peso (Prof: BIA)</v>
       </c>
       <c r="C41" t="str">
-        <v>Revisão</v>
+        <v>Condução do Paulista (Prof: DAVIDSON)</v>
       </c>
       <c r="D41" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>Passo de Cintura (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E41" t="str">
-        <v>Combinação de Cintura</v>
+        <v>Sacada/Meia-lua (Prof: GÃO)</v>
       </c>
       <c r="F41" t="str">
-        <v>Combinação de Cintura</v>
+        <v>giro completo (Prof: MESSIAS)</v>
       </c>
       <c r="G41" t="str">
-        <v>Revisão</v>
+        <v>passo de perna (Prof: GÃO)</v>
       </c>
       <c r="H41" t="str">
-        <v>Variações Giro do Condutor</v>
+        <v>Revisão (Prof: TAZ)</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Condução do Paulista (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>sábado, 11/10</v>
+        <v>sábado, 10/10</v>
       </c>
       <c r="B42" t="str">
-        <v>Leque</v>
+        <v>Meio Giro Trás/Frente (Aulão/Junto) (Prof: BIA)</v>
       </c>
       <c r="C42" t="str">
-        <v>Nivelamento</v>
+        <v>Movimentações do paulista (saída do pião/meio giro trás e do meio invertido trás) (Prof: DAVIDSON)</v>
       </c>
       <c r="D42" t="str">
-        <v>Chuveirinho</v>
+        <v>Esmeril junto (Prof: TONY E JULY)</v>
       </c>
       <c r="E42" t="str">
-        <v>Esmeril Fechado</v>
+        <v>Pêndulo/Ciscada (Prof: GÃO)</v>
       </c>
       <c r="F42" t="str">
-        <v>Esmeril Fechado</v>
+        <v>Meio Giro Trás/Frente (Aulão/Junto) (Prof: MESSIAS)</v>
       </c>
       <c r="G42" t="str">
-        <v>Nivelamento</v>
+        <v>Contratempo (Prof: GÃO)</v>
       </c>
       <c r="H42" t="str">
-        <v>Chuveirinho</v>
+        <v>Nivelamento (Prof: TAZ)</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Movimentações do paulista (saída do pião/meio giro trás e do meio invertido trás) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>sábado, 18/10</v>
+        <v>sábado, 17/10</v>
       </c>
       <c r="B43" t="str">
-        <v>Push and Pull</v>
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: BIA)</v>
       </c>
       <c r="C43" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
       <c r="D43" t="str">
-        <v>Manivela</v>
+        <v>Especial (Prof: TONY E JULY)</v>
       </c>
       <c r="E43" t="str">
-        <v>Práticas dançantes</v>
+        <v>Especial (Prof: GÃO)</v>
       </c>
       <c r="F43" t="str">
-        <v>Práticas dançantes</v>
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G43" t="str">
-        <v>Revisão de Contratempo</v>
+        <v>Especial (Prof: GÃO)</v>
       </c>
       <c r="H43" t="str">
-        <v>Manivela</v>
+        <v>invertido (Prof: TAZ)</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Pião invertido a partir do giro simples (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>sábado, 25/10</v>
+        <v>sábado, 24/10</v>
       </c>
       <c r="B44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Postura e Ritmo (Prof: BIA)</v>
       </c>
       <c r="C44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
       <c r="D44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Turma Junta (Prof: TONY E JULY)</v>
       </c>
       <c r="E44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Turma Junta (Prof: GÃO)</v>
       </c>
       <c r="F44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Postura e Ritmo (Prof: MESSIAS)</v>
       </c>
       <c r="G44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>Turma Junta (Prof: GÃO)</v>
       </c>
       <c r="H44" t="str">
-        <v>Halloween - AULA ESPECIAL</v>
+        <v>invertido + giro gira (Prof: TAZ)</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Pião invertido a partir do passo de cintura com contratempo 2 (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>sábado, 01/11</v>
+        <v>sábado, 31/10</v>
       </c>
       <c r="B45" t="str">
-        <v>Paulista Titanic</v>
+        <v>Giro Simples Cavalheiro/Dama (Prof: BIA)</v>
       </c>
       <c r="C45" t="str">
-        <v>Banana c contra</v>
+        <v>Variação de Avião (Prof: DAVIDSON)</v>
       </c>
       <c r="D45" t="str">
-        <v>Caracol</v>
+        <v>Meio Giro Invertido Trás/Frente (Aulão/Junto) (Prof: TONY E JULY)</v>
       </c>
       <c r="E45" t="str">
-        <v>Introdução Contratempo</v>
+        <v>Pião (Prof: GÃO)</v>
       </c>
       <c r="F45" t="str">
-        <v>Introdução Contratempo</v>
+        <v>Giro Simples Cavalheiro/Dama (Prof: MESSIAS)</v>
       </c>
       <c r="G45" t="str">
-        <v>Banana c contra</v>
+        <v>Pião (Prof: GÃO)</v>
       </c>
       <c r="H45" t="str">
-        <v>Caracol</v>
+        <v>Meio Giro Invertido Trás/Frente (Aulão/Junto) (Prof: TAZ)</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Variação de Avião (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>sábado, 08/11</v>
+        <v>sábado, 07/11</v>
       </c>
       <c r="B46" t="str">
-        <v>Contra 9 tempos</v>
+        <v>Peso e Contrapeso (Prof: BIA)</v>
       </c>
       <c r="C46" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>Contratempos duplos (sinistro e 1ª evolução do sinistro) (Prof: DAVIDSON)</v>
       </c>
       <c r="D46" t="str">
-        <v>Revisão</v>
+        <v>Avião (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E46" t="str">
-        <v>Caracol c Contra</v>
+        <v>Sinistro (Prof: GÃO)</v>
       </c>
       <c r="F46" t="str">
-        <v>Caracol c Contra</v>
+        <v>Peso e Contrapeso (Prof: MESSIAS)</v>
       </c>
       <c r="G46" t="str">
-        <v>Chuveirinho c Contra</v>
+        <v>Sinistro (Prof: GÃO)</v>
       </c>
       <c r="H46" t="str">
-        <v>Revisão</v>
+        <v>Avião (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Contratempos duplos (sinistro e 1ª evolução do sinistro) (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>sábado, 15/11</v>
+        <v>sábado, 14/11</v>
       </c>
       <c r="B47" t="str">
-        <v>Banana 9 tempos</v>
+        <v>Chameguinho (Aulão) (Prof: BIA)</v>
       </c>
       <c r="C47" t="str">
-        <v>Sinistro</v>
+        <v>Variação de Banana (Prof: DAVIDSON)</v>
       </c>
       <c r="D47" t="str">
-        <v>Nivelamento</v>
+        <v>Musicalidade (Prof: TONY E JULY)</v>
       </c>
       <c r="E47" t="str">
-        <v>Conduções de Contra</v>
+        <v>Contratempo (Prof: GÃO)</v>
       </c>
       <c r="F47" t="str">
-        <v>Conduções de Contra</v>
+        <v>Chameguinho (Aulão) (Prof: MESSIAS)</v>
       </c>
       <c r="G47" t="str">
-        <v>Sinistro</v>
+        <v>Contratempo (Prof: GÃO)</v>
       </c>
       <c r="H47" t="str">
-        <v>Nivelamento</v>
+        <v>Musicalidade (Prof: TAZ)</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Variação de Banana (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>sábado, 22/11</v>
+        <v>sábado, 21/11</v>
       </c>
       <c r="B48" t="str">
-        <v>Chuveirinho 9 tempos</v>
+        <v>Especial (Prof: BIA)</v>
       </c>
       <c r="C48" t="str">
-        <v>Avião c contra</v>
+        <v>Variação de Passos de Cintura (Prof: DAVIDSON)</v>
       </c>
       <c r="D48" t="str">
-        <v>Passo Básico</v>
+        <v>Banana (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E48" t="str">
-        <v>Contra do Passo Básico</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F48" t="str">
-        <v>Contra do Passo Básico</v>
+        <v>Especial (Prof: MESSIAS)</v>
       </c>
       <c r="G48" t="str">
-        <v>Avião c contra</v>
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H48" t="str">
-        <v>Passo Básico</v>
+        <v>Banana (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Variação de Passos de Cintura (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>sábado, 29/11</v>
+        <v>sábado, 28/11</v>
       </c>
       <c r="B49" t="str">
-        <v>Sinistro 9 e 11</v>
+        <v>Turma Junta (Prof: BIA)</v>
       </c>
       <c r="C49" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>Combinação de Cintura com Peões (Prof: DAVIDSON)</v>
       </c>
       <c r="D49" t="str">
-        <v>Xaxadinho</v>
+        <v>Chuveirinho (+Variações sem Contratempo (Prof: TONY E JULY)</v>
       </c>
       <c r="E49" t="str">
-        <v>Combinações de Contra</v>
+        <v>Banana (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F49" t="str">
-        <v>Combinações de Contra</v>
+        <v>Turma Junta (Prof: MESSIAS)</v>
       </c>
       <c r="G49" t="str">
-        <v>Contratempo DE 7 TEMPOS</v>
+        <v>Banana (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H49" t="str">
-        <v>Xaxadinho</v>
+        <v>Chuveirinho (+Variações sem Contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Combinação de Cintura com Peões (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>sábado, 06/12</v>
+        <v>sábado, 05/12</v>
       </c>
       <c r="B50" t="str">
-        <v>Avião Invertido</v>
+        <v>Passo Básico (Prof: BIA)</v>
       </c>
       <c r="C50" t="str">
-        <v>Basquete com Contra</v>
+        <v>Giros invertidos completos (Prof: DAVIDSON)</v>
       </c>
       <c r="D50" t="str">
-        <v>Deslocamento 1</v>
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
       </c>
       <c r="E50" t="str">
-        <v>Revisão</v>
+        <v>Giro completo trás/frente (junto) (Prof: GÃO)</v>
       </c>
       <c r="F50" t="str">
-        <v>Revisão</v>
+        <v>Passo Básico (Prof: MESSIAS)</v>
       </c>
       <c r="G50" t="str">
-        <v>Basquete com Contra</v>
+        <v>Giro completo trás/frente (junto) (Prof: GÃO)</v>
       </c>
       <c r="H50" t="str">
-        <v>Deslocamento 1</v>
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Giros invertidos completos (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>sábado, 13/12</v>
+        <v>sábado, 12/12</v>
       </c>
       <c r="B51" t="str">
-        <v>Beyblade 9</v>
+        <v>Soltinho (Prof: BIA)</v>
       </c>
       <c r="C51" t="str">
-        <v>Esmeril aberto</v>
+        <v>Esmeril unilateral (Prof: DAVIDSON)</v>
       </c>
       <c r="D51" t="str">
-        <v>Deslocamento 2</v>
+        <v>Caminhada Esquerda/Direita (Prof: TONY E JULY)</v>
       </c>
       <c r="E51" t="str">
-        <v>Nivelamento</v>
+        <v>Chuveirinho (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="F51" t="str">
-        <v>Nivelamento</v>
+        <v>Soltinho (Prof: MESSIAS)</v>
       </c>
       <c r="G51" t="str">
-        <v>Esmeril aberto</v>
+        <v>Chuveirinho (+Variações com Contratempo) (Prof: GÃO)</v>
       </c>
       <c r="H51" t="str">
-        <v>Deslocamento 2</v>
+        <v>Caminhada Esquerda/Direita (Prof: TAZ)</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Esmeril unilateral (Prof: DAVIDSON)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>sábado, 20/12</v>
+        <v>sábado, 19/12</v>
       </c>
       <c r="B52" t="str">
-        <v>Giro Simples 9 e 11</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="C52" t="str">
-        <v>Esmeril unilateral</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="D52" t="str">
-        <v>Ritmos</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="E52" t="str">
-        <v>Ritmo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="F52" t="str">
-        <v>Ritmo</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="G52" t="str">
-        <v>Esmeril unilateral</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="H52" t="str">
-        <v>Ritmos</v>
+        <v>SEM AULA - RECESSO</v>
+      </c>
+      <c r="I52" t="str">
+        <v>SEM AULA - RECESSO</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>sábado, 27/12</v>
+        <v>sábado, 26/12</v>
       </c>
       <c r="B53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="C53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="D53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="E53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="F53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="G53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
       </c>
       <c r="H53" t="str">
-        <v>NATAL - Sem aula</v>
+        <v>SEM AULA - RECESSO</v>
+      </c>
+      <c r="I53" t="str">
+        <v>SEM AULA - RECESSO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I53"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I52"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Data</v>
+      </c>
+      <c r="B1" t="str">
+        <v>B1 Manhã</v>
+      </c>
+      <c r="C1" t="str">
+        <v>I2 Manhã</v>
+      </c>
+      <c r="D1" t="str">
+        <v>B2 Manhã</v>
+      </c>
+      <c r="E1" t="str">
+        <v>I1 Manhã</v>
+      </c>
+      <c r="F1" t="str">
+        <v>B1 Tarde</v>
+      </c>
+      <c r="G1" t="str">
+        <v>I1 Tarde</v>
+      </c>
+      <c r="H1" t="str">
+        <v>B2 Tarde</v>
+      </c>
+      <c r="I1" t="str">
+        <v>I2 Tarde</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>sábado, 07/01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Aula com BIA</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Turma junta (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Musicalidade (Prof: TONY)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Sacada/Meia-lua (Prof: DAVIDSON)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Aula com MESSIAS</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Passo de Cintura (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sábado, 14/01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Aula com BIA</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Passo de perna (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Especial (Prof: TONY E JULY)</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Aula com GÃO</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Meio Giro Trás/Frente (Aulão/Junto) (Prof: MESSIAS)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Passo de Cintura (+Variações sem Contratempo) (Prof: TAZ)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>sábado, 21/01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Giro Completo Trás/Frente (Aulão) (Prof: BIA)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sequência de passo de perna + paulista (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Giro-Giro (+Variações sem Contratempo) (Prof: TONY E JULY)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sequência de caracol com avião (Prof: GÃO)</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Revisão passo simples, soltinho e meio giro (Prof: MESSIAS)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Avião (+Variações com Contratempo) (Prof: GÃO)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Revisão passo cintura e início esmeril (Prof: TAZ)</v>
+      </c>
+      <c r="I4" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>sábado, 28/01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Abertura soltinho e giro simples (Prof: BIA)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Avião invertido + contratempo (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Giro-giro (Prof: GÃO)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Avião com contratempos (Prof: GÃO)</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Meio giro (Prof: MESSIAS)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>—</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Esmeril junto (Prof: TAZ)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>sábado, 04/02</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Troca de peso e passo básico (Prof: BIA)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sequência das últimas aulas (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Banana banana (Prof: TONY)</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Avião + contratempo (Prof: TAZ E BIA)</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Passo básico e meio-giros (Prof: BIA)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Giro-giro com contratempo (Prof: TAZ E BIA)</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Esmeril junto (Prof: TAZ E JULY)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>sábado, 11/02</v>
+      </c>
+      <c r="B7" t="str">
+        <v>—</v>
+      </c>
+      <c r="C7" t="str">
+        <v>—</v>
+      </c>
+      <c r="D7" t="str">
+        <v>—</v>
+      </c>
+      <c r="E7" t="str">
+        <v>—</v>
+      </c>
+      <c r="F7" t="str">
+        <v>—</v>
+      </c>
+      <c r="G7" t="str">
+        <v>—</v>
+      </c>
+      <c r="H7" t="str">
+        <v>—</v>
+      </c>
+      <c r="I7" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>sábado, 25/02</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Giro da dama e giro cavalheiro (Prof: JULY)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>—</v>
+      </c>
+      <c r="D8" t="str">
+        <v>banana-banana (Prof: DAVIDSON)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>turma junta (Prof: DAVIDSON)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>básico e meio-giro (Prof: JULY)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>chuveirinho com contratempo + banana com contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Início contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I8" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>sábado, 04/03</v>
+      </c>
+      <c r="B9" t="str">
+        <v>GIRO SIMPLES (Prof: BIA)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Sequencia com contratempo de 7 (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Avião (Prof: TONY)</v>
+      </c>
+      <c r="E9" t="str">
+        <v>giro-giro com contratempo (Prof: GÃO)</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Postura + passos iniciais (Prof: MESSIAS)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>contratempo de 5 tempos + 7 tempos (Prof: GÃO)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>CONTRATEMPO condução (Prof: TAZ E JULY)</v>
+      </c>
+      <c r="I9" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>sábado, 11/03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>xaxadinho; chuveirinho (Prof: GÃO)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Introdução cretinagem (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Revisão (Prof: TONY)</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Aula com GÃO</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Giro simples (Prof: JULY)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>sinistro com contratempo + banana invertida (Prof: GÃO)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>contratempo (Prof: TONY)</v>
+      </c>
+      <c r="I10" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>sábado, 18/03</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Meios giros/Nivelamento (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Giro completo invertido + pião invertido (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Início de cintura (Prof: TONY)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Aula com GÃO E BIA</v>
+      </c>
+      <c r="F11" t="str">
+        <v>GIro simples</v>
+      </c>
+      <c r="G11" t="str">
+        <v>—</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Caracol com contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I11" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>sábado, 25/03</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Início Módulo</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Sacada com a perna esquerda (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>passo de cintura (Prof: TONY)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>—</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Giro simples (Prof: JULY)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Introdução Paulista (Prof: GÃO)</v>
+      </c>
+      <c r="H12" t="str">
+        <v>REVISÃO (Prof: TAZ)</v>
+      </c>
+      <c r="I12" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>sábado, 01/04</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Peso e contrapeso (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Sacada de letra (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>passo de cintura (Prof: TONY)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Introdução ao Paulista (Prof: GÃO)</v>
+      </c>
+      <c r="F13" t="str">
+        <v>—</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Paulista com invertido atrás (Prof: GÃO)</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Revisão Nivelamento (Prof: TAZ)</v>
+      </c>
+      <c r="I13" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>sábado, 08/04</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Meio-giro dançando junto (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Sequencia de sacada de esquerda (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Passo de cintura saindo no invertido (Prof: TONY E JULY)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Paulista (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Giro do cavalheiro (Prof: MESSIAS)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Paulista (Prof: GÃO)</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Revisão e Nivelamento (Prof: TAZ)</v>
+      </c>
+      <c r="I14" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>sábado, 15/04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>—</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Aula livre (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Ritmo (Prof: TONY)</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Nivelamento + Paulista (Prof: GÃO)</v>
+      </c>
+      <c r="F15" t="str">
+        <v>—</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Banana finalizando com paulista (Prof: GÃO)</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Aula junto com o Básico 1</v>
+      </c>
+      <c r="I15" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>sábado, 22/04</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Revisão (Prof: BIA)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>bêbado (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>ESMERIL JUNTO</v>
+      </c>
+      <c r="E16" t="str">
+        <v>PAULISTA COM INVERTIDO TRÁS (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Variação do giro simples (Prof: JULY)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>introdução ao esmeril (Prof: GÃO E JULY)</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Revisão (Prof: TAZ)</v>
+      </c>
+      <c r="I16" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>sábado, 29/04</v>
+      </c>
+      <c r="B17" t="str">
+        <v>variações de giro simples (Prof: BIA)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>paulista (Prof: DAVIDSON)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>esmeril junto (Prof: TONY)</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Paulista com invertido (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F17" t="str">
+        <v>—</v>
+      </c>
+      <c r="G17" t="str">
+        <v>esmeril (variações) (Prof: GÃO)</v>
+      </c>
+      <c r="H17" t="str">
+        <v>—</v>
+      </c>
+      <c r="I17" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>sábado, 06/05</v>
+      </c>
+      <c r="B18" t="str">
+        <v>—</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Aula com DAVIDSON</v>
+      </c>
+      <c r="D18" t="str">
+        <v>esmeril (Prof: DAVIDSON)</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Introdução esmeril aberto (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F18" t="str">
+        <v>—</v>
+      </c>
+      <c r="G18" t="str">
+        <v>esmeril; introdução pião (Prof: GÃO)</v>
+      </c>
+      <c r="H18" t="str">
+        <v>NIVELAMENTO</v>
+      </c>
+      <c r="I18" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>sábado, 13/05</v>
+      </c>
+      <c r="B19" t="str">
+        <v>REVISÃO</v>
+      </c>
+      <c r="C19" t="str">
+        <v>—</v>
+      </c>
+      <c r="D19" t="str">
+        <v>cobrinha</v>
+      </c>
+      <c r="E19" t="str">
+        <v>esmeril abberto</v>
+      </c>
+      <c r="F19" t="str">
+        <v>manivela</v>
+      </c>
+      <c r="G19" t="str">
+        <v>pião</v>
+      </c>
+      <c r="H19" t="str">
+        <v>invertido</v>
+      </c>
+      <c r="I19" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>sábado, 20/05</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Nivelamento</v>
+      </c>
+      <c r="C20" t="str">
+        <v>—</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Contratempo introdução</v>
+      </c>
+      <c r="E20" t="str">
+        <v>esmeril variações</v>
+      </c>
+      <c r="F20" t="str">
+        <v>nivelamento</v>
+      </c>
+      <c r="G20" t="str">
+        <v>pião</v>
+      </c>
+      <c r="H20" t="str">
+        <v>revisão</v>
+      </c>
+      <c r="I20" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>sábado, 27/05</v>
+      </c>
+      <c r="B21" t="str">
+        <v>—</v>
+      </c>
+      <c r="C21" t="str">
+        <v>—</v>
+      </c>
+      <c r="D21" t="str">
+        <v>contratempo (Prof: TONY)</v>
+      </c>
+      <c r="E21" t="str">
+        <v>técnicas de esmeril (Prof: BIA)</v>
+      </c>
+      <c r="F21" t="str">
+        <v>—</v>
+      </c>
+      <c r="G21" t="str">
+        <v>técnicas de esmeril (Prof: BIA)</v>
+      </c>
+      <c r="H21" t="str">
+        <v>—</v>
+      </c>
+      <c r="I21" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>sábado, 03/06</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Aula com BIA</v>
+      </c>
+      <c r="C22" t="str">
+        <v>—</v>
+      </c>
+      <c r="D22" t="str">
+        <v>contratempo (Prof: TONY)</v>
+      </c>
+      <c r="E22" t="str">
+        <v>I1 e I2 Pião (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F22" t="str">
+        <v>manivela, giro dama e cavalheiro, variações (Prof: MESSIAS)</v>
+      </c>
+      <c r="G22" t="str">
+        <v>pião invertido</v>
+      </c>
+      <c r="H22" t="str">
+        <v>combo de giro (Prof: TAZ)</v>
+      </c>
+      <c r="I22" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>sábado, 10/06</v>
+      </c>
+      <c r="B23" t="str">
+        <v>—</v>
+      </c>
+      <c r="C23" t="str">
+        <v>—</v>
+      </c>
+      <c r="D23" t="str">
+        <v>contratempo</v>
+      </c>
+      <c r="E23" t="str">
+        <v>pião</v>
+      </c>
+      <c r="F23" t="str">
+        <v>giro do cavalheiro</v>
+      </c>
+      <c r="G23" t="str">
+        <v>pião + contratempo</v>
+      </c>
+      <c r="H23" t="str">
+        <v>banana-banana</v>
+      </c>
+      <c r="I23" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>sábado, 17/06</v>
+      </c>
+      <c r="B24" t="str">
+        <v>—</v>
+      </c>
+      <c r="C24" t="str">
+        <v>—</v>
+      </c>
+      <c r="D24" t="str">
+        <v>contratempo</v>
+      </c>
+      <c r="E24" t="str">
+        <v>pião</v>
+      </c>
+      <c r="F24" t="str">
+        <v>—</v>
+      </c>
+      <c r="G24" t="str">
+        <v>pião com travada</v>
+      </c>
+      <c r="H24" t="str">
+        <v>avião</v>
+      </c>
+      <c r="I24" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>sábado, 24/06</v>
+      </c>
+      <c r="B25" t="str">
+        <v>—</v>
+      </c>
+      <c r="C25" t="str">
+        <v>—</v>
+      </c>
+      <c r="D25" t="str">
+        <v>—</v>
+      </c>
+      <c r="E25" t="str">
+        <v>—</v>
+      </c>
+      <c r="F25" t="str">
+        <v>—</v>
+      </c>
+      <c r="G25" t="str">
+        <v>—</v>
+      </c>
+      <c r="H25" t="str">
+        <v>—</v>
+      </c>
+      <c r="I25" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>sábado, 01/07</v>
+      </c>
+      <c r="B26" t="str">
+        <v>—</v>
+      </c>
+      <c r="C26" t="str">
+        <v>—</v>
+      </c>
+      <c r="D26" t="str">
+        <v>—</v>
+      </c>
+      <c r="E26" t="str">
+        <v>pião</v>
+      </c>
+      <c r="F26" t="str">
+        <v>—</v>
+      </c>
+      <c r="G26" t="str">
+        <v>sacada de perna</v>
+      </c>
+      <c r="H26" t="str">
+        <v>—</v>
+      </c>
+      <c r="I26" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>sábado, 08/07</v>
+      </c>
+      <c r="B27" t="str">
+        <v>peso e contrapeso (Prof: BIA)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>—</v>
+      </c>
+      <c r="D27" t="str">
+        <v>contratempo (Prof: TONY)</v>
+      </c>
+      <c r="E27" t="str">
+        <v>—</v>
+      </c>
+      <c r="F27" t="str">
+        <v>—</v>
+      </c>
+      <c r="G27" t="str">
+        <v>—</v>
+      </c>
+      <c r="H27" t="str">
+        <v>—</v>
+      </c>
+      <c r="I27" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>sábado, 15/07</v>
+      </c>
+      <c r="B28" t="str">
+        <v>musicalidade</v>
+      </c>
+      <c r="C28" t="str">
+        <v>-</v>
+      </c>
+      <c r="D28" t="str">
+        <v>contratempo</v>
+      </c>
+      <c r="E28" t="str">
+        <v>pião com travada</v>
+      </c>
+      <c r="F28" t="str">
+        <v>—</v>
+      </c>
+      <c r="G28" t="str">
+        <v>caminhada e travada</v>
+      </c>
+      <c r="H28" t="str">
+        <v>—</v>
+      </c>
+      <c r="I28" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>sábado, 22/07</v>
+      </c>
+      <c r="B29" t="str">
+        <v>—</v>
+      </c>
+      <c r="C29" t="str">
+        <v>—</v>
+      </c>
+      <c r="D29" t="str">
+        <v>—</v>
+      </c>
+      <c r="E29" t="str">
+        <v>—</v>
+      </c>
+      <c r="F29" t="str">
+        <v>—</v>
+      </c>
+      <c r="G29" t="str">
+        <v>—</v>
+      </c>
+      <c r="H29" t="str">
+        <v>—</v>
+      </c>
+      <c r="I29" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>sábado, 29/07</v>
+      </c>
+      <c r="B30" t="str">
+        <v>—</v>
+      </c>
+      <c r="C30" t="str">
+        <v>—</v>
+      </c>
+      <c r="D30" t="str">
+        <v>—</v>
+      </c>
+      <c r="E30" t="str">
+        <v>—</v>
+      </c>
+      <c r="F30" t="str">
+        <v>—</v>
+      </c>
+      <c r="G30" t="str">
+        <v>—</v>
+      </c>
+      <c r="H30" t="str">
+        <v>—</v>
+      </c>
+      <c r="I30" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>sábado, 05/08</v>
+      </c>
+      <c r="B31" t="str">
+        <v>—</v>
+      </c>
+      <c r="C31" t="str">
+        <v>—</v>
+      </c>
+      <c r="D31" t="str">
+        <v>invertido (Prof: TONY)</v>
+      </c>
+      <c r="E31" t="str">
+        <v>caminhada + variações (Prof: GÃO E BIA)</v>
+      </c>
+      <c r="F31" t="str">
+        <v>-</v>
+      </c>
+      <c r="G31" t="str">
+        <v>—</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Aula com TAZ</v>
+      </c>
+      <c r="I31" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>sábado, 12/08</v>
+      </c>
+      <c r="B32" t="str">
+        <v>—</v>
+      </c>
+      <c r="C32" t="str">
+        <v>—</v>
+      </c>
+      <c r="D32" t="str">
+        <v>—</v>
+      </c>
+      <c r="E32" t="str">
+        <v>—</v>
+      </c>
+      <c r="F32" t="str">
+        <v>—</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Aula com GÃO</v>
+      </c>
+      <c r="H32" t="str">
+        <v>início de contratempo (Prof: TAZ)</v>
+      </c>
+      <c r="I32" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>sábado, 19/08</v>
+      </c>
+      <c r="B33" t="str">
+        <v>—</v>
+      </c>
+      <c r="C33" t="str">
+        <v>—</v>
+      </c>
+      <c r="D33" t="str">
+        <v>invertido</v>
+      </c>
+      <c r="E33" t="str">
+        <v>breck</v>
+      </c>
+      <c r="F33" t="str">
+        <v>—</v>
+      </c>
+      <c r="G33" t="str">
+        <v>—</v>
+      </c>
+      <c r="H33" t="str">
+        <v>contratempo</v>
+      </c>
+      <c r="I33" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>sábado, 26/08</v>
+      </c>
+      <c r="B34" t="str">
+        <v>—</v>
+      </c>
+      <c r="C34" t="str">
+        <v>—</v>
+      </c>
+      <c r="D34" t="str">
+        <v>—</v>
+      </c>
+      <c r="E34" t="str">
+        <v>—</v>
+      </c>
+      <c r="F34" t="str">
+        <v>—</v>
+      </c>
+      <c r="G34" t="str">
+        <v>—</v>
+      </c>
+      <c r="H34" t="str">
+        <v>—</v>
+      </c>
+      <c r="I34" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>sábado, 02/09</v>
+      </c>
+      <c r="B35" t="str">
+        <v>—</v>
+      </c>
+      <c r="C35" t="str">
+        <v>—</v>
+      </c>
+      <c r="D35" t="str">
+        <v>—</v>
+      </c>
+      <c r="E35" t="str">
+        <v>—</v>
+      </c>
+      <c r="F35" t="str">
+        <v>—</v>
+      </c>
+      <c r="G35" t="str">
+        <v>—</v>
+      </c>
+      <c r="H35" t="str">
+        <v>—</v>
+      </c>
+      <c r="I35" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>sábado, 09/09</v>
+      </c>
+      <c r="B36" t="str">
+        <v>—</v>
+      </c>
+      <c r="C36" t="str">
+        <v>—</v>
+      </c>
+      <c r="D36" t="str">
+        <v>—</v>
+      </c>
+      <c r="E36" t="str">
+        <v>—</v>
+      </c>
+      <c r="F36" t="str">
+        <v>—</v>
+      </c>
+      <c r="G36" t="str">
+        <v>—</v>
+      </c>
+      <c r="H36" t="str">
+        <v>—</v>
+      </c>
+      <c r="I36" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>sábado, 16/09</v>
+      </c>
+      <c r="B37" t="str">
+        <v>—</v>
+      </c>
+      <c r="C37" t="str">
+        <v>—</v>
+      </c>
+      <c r="D37" t="str">
+        <v>—</v>
+      </c>
+      <c r="E37" t="str">
+        <v>—</v>
+      </c>
+      <c r="F37" t="str">
+        <v>giro completo</v>
+      </c>
+      <c r="G37" t="str">
+        <v>passo de perna</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Revisão</v>
+      </c>
+      <c r="I37" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>sábado, 23/09</v>
+      </c>
+      <c r="B38" t="str">
+        <v>—</v>
+      </c>
+      <c r="C38" t="str">
+        <v>—</v>
+      </c>
+      <c r="D38" t="str">
+        <v>—</v>
+      </c>
+      <c r="E38" t="str">
+        <v>—</v>
+      </c>
+      <c r="F38" t="str">
+        <v>—</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Contratempo</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Nivelamento</v>
+      </c>
+      <c r="I38" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>sábado, 30/09</v>
+      </c>
+      <c r="B39" t="str">
+        <v>—</v>
+      </c>
+      <c r="C39" t="str">
+        <v>—</v>
+      </c>
+      <c r="D39" t="str">
+        <v>—</v>
+      </c>
+      <c r="E39" t="str">
+        <v>—</v>
+      </c>
+      <c r="F39" t="str">
+        <v>—</v>
+      </c>
+      <c r="G39" t="str">
+        <v>—</v>
+      </c>
+      <c r="H39" t="str">
+        <v>invertido</v>
+      </c>
+      <c r="I39" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>sábado, 07/10</v>
+      </c>
+      <c r="B40" t="str">
+        <v>—</v>
+      </c>
+      <c r="C40" t="str">
+        <v>—</v>
+      </c>
+      <c r="D40" t="str">
+        <v>—</v>
+      </c>
+      <c r="E40" t="str">
+        <v>—</v>
+      </c>
+      <c r="F40" t="str">
+        <v>—</v>
+      </c>
+      <c r="G40" t="str">
+        <v>—</v>
+      </c>
+      <c r="H40" t="str">
+        <v>invertido + giro gira</v>
+      </c>
+      <c r="I40" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>sábado, 14/10</v>
+      </c>
+      <c r="B41" t="str">
+        <v>—</v>
+      </c>
+      <c r="C41" t="str">
+        <v>—</v>
+      </c>
+      <c r="D41" t="str">
+        <v>—</v>
+      </c>
+      <c r="E41" t="str">
+        <v>—</v>
+      </c>
+      <c r="F41" t="str">
+        <v>—</v>
+      </c>
+      <c r="G41" t="str">
+        <v>—</v>
+      </c>
+      <c r="H41" t="str">
+        <v>—</v>
+      </c>
+      <c r="I41" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>sábado, 21/10</v>
+      </c>
+      <c r="B42" t="str">
+        <v>—</v>
+      </c>
+      <c r="C42" t="str">
+        <v>—</v>
+      </c>
+      <c r="D42" t="str">
+        <v>—</v>
+      </c>
+      <c r="E42" t="str">
+        <v>—</v>
+      </c>
+      <c r="F42" t="str">
+        <v>—</v>
+      </c>
+      <c r="G42" t="str">
+        <v>—</v>
+      </c>
+      <c r="H42" t="str">
+        <v>—</v>
+      </c>
+      <c r="I42" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>sábado, 28/10</v>
+      </c>
+      <c r="B43" t="str">
+        <v>—</v>
+      </c>
+      <c r="C43" t="str">
+        <v>—</v>
+      </c>
+      <c r="D43" t="str">
+        <v>—</v>
+      </c>
+      <c r="E43" t="str">
+        <v>—</v>
+      </c>
+      <c r="F43" t="str">
+        <v>—</v>
+      </c>
+      <c r="G43" t="str">
+        <v>—</v>
+      </c>
+      <c r="H43" t="str">
+        <v>—</v>
+      </c>
+      <c r="I43" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>sábado, 04/11</v>
+      </c>
+      <c r="B44" t="str">
+        <v>—</v>
+      </c>
+      <c r="C44" t="str">
+        <v>—</v>
+      </c>
+      <c r="D44" t="str">
+        <v>—</v>
+      </c>
+      <c r="E44" t="str">
+        <v>—</v>
+      </c>
+      <c r="F44" t="str">
+        <v>—</v>
+      </c>
+      <c r="G44" t="str">
+        <v>—</v>
+      </c>
+      <c r="H44" t="str">
+        <v>—</v>
+      </c>
+      <c r="I44" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>sábado, 11/11</v>
+      </c>
+      <c r="B45" t="str">
+        <v>—</v>
+      </c>
+      <c r="C45" t="str">
+        <v>—</v>
+      </c>
+      <c r="D45" t="str">
+        <v>—</v>
+      </c>
+      <c r="E45" t="str">
+        <v>—</v>
+      </c>
+      <c r="F45" t="str">
+        <v>—</v>
+      </c>
+      <c r="G45" t="str">
+        <v>—</v>
+      </c>
+      <c r="H45" t="str">
+        <v>—</v>
+      </c>
+      <c r="I45" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>sábado, 18/11</v>
+      </c>
+      <c r="B46" t="str">
+        <v>—</v>
+      </c>
+      <c r="C46" t="str">
+        <v>—</v>
+      </c>
+      <c r="D46" t="str">
+        <v>—</v>
+      </c>
+      <c r="E46" t="str">
+        <v>—</v>
+      </c>
+      <c r="F46" t="str">
+        <v>—</v>
+      </c>
+      <c r="G46" t="str">
+        <v>—</v>
+      </c>
+      <c r="H46" t="str">
+        <v>—</v>
+      </c>
+      <c r="I46" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>sábado, 25/11</v>
+      </c>
+      <c r="B47" t="str">
+        <v>—</v>
+      </c>
+      <c r="C47" t="str">
+        <v>—</v>
+      </c>
+      <c r="D47" t="str">
+        <v>—</v>
+      </c>
+      <c r="E47" t="str">
+        <v>—</v>
+      </c>
+      <c r="F47" t="str">
+        <v>—</v>
+      </c>
+      <c r="G47" t="str">
+        <v>—</v>
+      </c>
+      <c r="H47" t="str">
+        <v>—</v>
+      </c>
+      <c r="I47" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>sábado, 02/12</v>
+      </c>
+      <c r="B48" t="str">
+        <v>—</v>
+      </c>
+      <c r="C48" t="str">
+        <v>—</v>
+      </c>
+      <c r="D48" t="str">
+        <v>—</v>
+      </c>
+      <c r="E48" t="str">
+        <v>—</v>
+      </c>
+      <c r="F48" t="str">
+        <v>—</v>
+      </c>
+      <c r="G48" t="str">
+        <v>—</v>
+      </c>
+      <c r="H48" t="str">
+        <v>—</v>
+      </c>
+      <c r="I48" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>sábado, 09/12</v>
+      </c>
+      <c r="B49" t="str">
+        <v>—</v>
+      </c>
+      <c r="C49" t="str">
+        <v>—</v>
+      </c>
+      <c r="D49" t="str">
+        <v>—</v>
+      </c>
+      <c r="E49" t="str">
+        <v>—</v>
+      </c>
+      <c r="F49" t="str">
+        <v>—</v>
+      </c>
+      <c r="G49" t="str">
+        <v>—</v>
+      </c>
+      <c r="H49" t="str">
+        <v>—</v>
+      </c>
+      <c r="I49" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>sábado, 16/12</v>
+      </c>
+      <c r="B50" t="str">
+        <v>—</v>
+      </c>
+      <c r="C50" t="str">
+        <v>—</v>
+      </c>
+      <c r="D50" t="str">
+        <v>—</v>
+      </c>
+      <c r="E50" t="str">
+        <v>—</v>
+      </c>
+      <c r="F50" t="str">
+        <v>—</v>
+      </c>
+      <c r="G50" t="str">
+        <v>—</v>
+      </c>
+      <c r="H50" t="str">
+        <v>—</v>
+      </c>
+      <c r="I50" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>sábado, 23/12</v>
+      </c>
+      <c r="B51" t="str">
+        <v>—</v>
+      </c>
+      <c r="C51" t="str">
+        <v>—</v>
+      </c>
+      <c r="D51" t="str">
+        <v>—</v>
+      </c>
+      <c r="E51" t="str">
+        <v>—</v>
+      </c>
+      <c r="F51" t="str">
+        <v>—</v>
+      </c>
+      <c r="G51" t="str">
+        <v>—</v>
+      </c>
+      <c r="H51" t="str">
+        <v>—</v>
+      </c>
+      <c r="I51" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>sábado, 30/12</v>
+      </c>
+      <c r="B52" t="str">
+        <v>—</v>
+      </c>
+      <c r="C52" t="str">
+        <v>—</v>
+      </c>
+      <c r="D52" t="str">
+        <v>—</v>
+      </c>
+      <c r="E52" t="str">
+        <v>—</v>
+      </c>
+      <c r="F52" t="str">
+        <v>—</v>
+      </c>
+      <c r="G52" t="str">
+        <v>—</v>
+      </c>
+      <c r="H52" t="str">
+        <v>—</v>
+      </c>
+      <c r="I52" t="str">
+        <v>—</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>